<commit_message>
Fix HS pitcher stats and unify summer season toggles across tabs.
Restore MaxPreps pitching extraction, correct pitcher/two-way roles, move overlapping AR follow players to the HS client list, and add visible school vs summer stat switching on HS, amateur, and watch list views.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/client_lists/ARFollow.xlsx
+++ b/client_lists/ARFollow.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -559,64 +559,56 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Cooper Vais</t>
+          <t>Luke Shoemaker</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>2027</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>RHP</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2027 USA Prime/Detroit Tigers Scout</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Arvada West HS</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Arvada</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>CO</t>
-        </is>
-      </c>
+          <t>2027 NorCal</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>https://www.maxpreps.com/co/arvada/arvada-west-wildcats/athletes/cooper-vais/baseball/stats/</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Gavin McMillan</t>
+          <t>Jaxxon Tweedt</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2027 Canes National</t>
+          <t>2028 Alpha Prime</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Monte Vista HS</t>
+          <t>Chico HS</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Danville</t>
+          <t>Chico</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -627,7 +619,7 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://www.maxpreps.com/ca/danville/monte-vista-mustangs/athletes/gavin-mcmillan/baseball/stats/</t>
+          <t>https://www.maxpreps.com/ca/chico/chico-panthers/athletes/jaxxon-tweedt/baseball/stats/</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -635,16 +627,20 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Luke Shoemaker</t>
+          <t>Miles Cornell</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2027</v>
-      </c>
-      <c r="C6" t="inlineStr"/>
+        <v>2028</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>RHP</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2027 NorCal</t>
+          <t>2028 Alpha Prime</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
@@ -661,7 +657,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Jaxxon Tweedt</t>
+          <t>Jack Carpenter</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -673,42 +669,34 @@
           <t>2028 Alpha Prime</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Chico HS</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Chico</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>https://www.maxpreps.com/ca/chico/chico-panthers/athletes/jaxxon-tweedt/baseball/stats/</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Miles Cornell</t>
+          <t>Austin Rider</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>2028</v>
       </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>RHP</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2028 Alpha Prime</t>
+          <t>2028 NorCal</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
@@ -725,16 +713,20 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Jack Carpenter</t>
+          <t>Chase Cotton</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>2028</v>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>RHP</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2028 Alpha Prime</t>
+          <t>2028 Canes National</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -742,16 +734,12 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Austin Rider</t>
+          <t>Brandon Williams</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -760,7 +748,7 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2028 NorCal</t>
+          <t>2028 MLB Breakthrough</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
@@ -768,47 +756,63 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Chase Cotton</t>
+          <t>Aiden Tavares</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2028 Canes National</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+          <t>2027 Top Tier</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Foothill HS</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Pleasanton</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://www.maxpreps.com/ca/pleasanton/foothill-falcons/athletes/aiden-taveres/baseball/stats/</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Brandon Williams</t>
+          <t>Michael Ohman</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2028</v>
-      </c>
-      <c r="C12" t="inlineStr"/>
+        <v>2029</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>LHP</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2028 MLB Breakthrough</t>
+          <t>2029 Alpha Prime</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
@@ -816,50 +820,42 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Aiden Tavares</t>
+          <t>Cole Callen</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2027</v>
+        <v>2029</v>
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2027 Top Tier</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Foothill HS</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Pleasanton</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
+          <t>2029 Alpha Prime</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>https://www.maxpreps.com/ca/pleasanton/foothill-falcons/athletes/aiden-taveres/baseball/stats/</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Enzi Otieku</t>
+          <t>Tommy Leeper</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -868,7 +864,7 @@
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2029 NorCal</t>
+          <t>2029 Alpha Prime</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
@@ -876,25 +872,25 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Michael Ohman</t>
+          <t>AJ Wida</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2029</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>LHP</t>
-        </is>
-      </c>
+        <v>2028</v>
+      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2029 Alpha Prime</t>
+          <t>2028 Franklin Scout</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
@@ -911,7 +907,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Cole Callen</t>
+          <t>Wyatt Gordon</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -920,7 +916,7 @@
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2029 Alpha Prime</t>
+          <t>2029 USA Prime National</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
@@ -937,7 +933,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Tommy Leeper</t>
+          <t>Damian Rivas</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -946,7 +942,7 @@
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2029 Alpha Prime</t>
+          <t>2029 USA Prime National</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -963,16 +959,16 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AJ Wida</t>
+          <t>Amani Tuiasosopo</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2028</v>
+        <v>2030</v>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2028 Franklin Scout</t>
+          <t>2030 USA Prime National</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
@@ -989,16 +985,16 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Wyatt Gordon</t>
+          <t>Brandon Sweeney</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2029</v>
+        <v>2030</v>
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2029 USA Prime National</t>
+          <t>2030 USA Prime National</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -1012,84 +1008,6 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Damian Rivas</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>2029</v>
-      </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>2029 USA Prime National</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Amani Tuiasosopo</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>2030</v>
-      </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>2030 USA Prime National</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Brandon Sweeney</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>2030</v>
-      </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>2030 USA Prime National</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix NorCal 2028 GC squad matching and add Jaxon Becker to AR follow.
Map NorCal U 2028 16U and LoForte with internal IDs, score squads by
recent/season volume instead of first roster hit, and stop broad GC
discovery when explicit program teams exist so Rider and Becker pull
from their active summer teams.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/client_lists/ARFollow.xlsx
+++ b/client_lists/ARFollow.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1008,6 +1008,36 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Jaxon Becker</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2028</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>RHP/1B</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2028 NorCal</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>